<commit_message>
Updated gitignore. Added support for lookups and Spool Detail Reference
</commit_message>
<xml_diff>
--- a/Joint Lookup.xlsx
+++ b/Joint Lookup.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmccall\source\repos\cmccall95\FabManager_To_QB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30B8142A-F6D7-497C-BCCC-685C51229171}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF9F0C09-8971-465B-9A92-E95D470829EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F2881F7C-457F-48D3-8FFD-7173B06AF8C8}"/>
+    <workbookView xWindow="-28920" yWindow="-1185" windowWidth="29040" windowHeight="15720" xr2:uid="{F2881F7C-457F-48D3-8FFD-7173B06AF8C8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>